<commit_message>
Scrap quotidien automatique (2026-09-07)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1021</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1028</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1021"/>
+  <dimension ref="A1:K1028"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48462,8 +48462,337 @@
         <v>36935881</v>
       </c>
     </row>
+    <row r="1022">
+      <c r="A1022" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1022" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1022" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1022" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1022" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1022" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1022" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1022" t="n">
+        <v>37240291</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1023" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1023" t="n">
+        <v>8</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1023" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="I1023" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1023" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1023" t="n">
+        <v>36336037</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1024" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1024" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1024" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1024" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1024" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1024" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1024" t="n">
+        <v>37240434</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1025" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1025" t="n">
+        <v>29</v>
+      </c>
+      <c r="G1025" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1025" t="inlineStr">
+        <is>
+          <t>29/36</t>
+        </is>
+      </c>
+      <c r="I1025" s="5" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="J1025" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1025" t="n">
+        <v>36892151</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1026" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1026" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1026" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1026" t="inlineStr">
+        <is>
+          <t>17/28</t>
+        </is>
+      </c>
+      <c r="I1026" s="5" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="J1026" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1026" t="n">
+        <v>36336252</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1027" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1027" t="n">
+        <v>30</v>
+      </c>
+      <c r="G1027" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1027" t="inlineStr">
+        <is>
+          <t>30/28</t>
+        </is>
+      </c>
+      <c r="I1027" s="3" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="J1027" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="K1027" t="n">
+        <v>36692764</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Dimanche</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1028" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1028" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1028" t="inlineStr">
+        <is>
+          <t>16/36</t>
+        </is>
+      </c>
+      <c r="I1028" s="4" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="J1028" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1028" t="n">
+        <v>36892106</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1021"/>
+  <autoFilter ref="A1:K1028"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-08)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1028</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1034</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1028"/>
+  <dimension ref="A1:K1034"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48791,8 +48791,290 @@
         <v>36892106</v>
       </c>
     </row>
+    <row r="1029">
+      <c r="A1029" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1029" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1029" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1029" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1029" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1029" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1029" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1029" t="n">
+        <v>36390338</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1030" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1030" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1030" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1030" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1030" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1030" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1030" t="n">
+        <v>38531917</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1031" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1031" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1031" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1031" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1031" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1031" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1031" t="n">
+        <v>36928736</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1032" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1032" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1032" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1032" t="inlineStr">
+        <is>
+          <t>15/28</t>
+        </is>
+      </c>
+      <c r="I1032" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J1032" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1032" t="n">
+        <v>36281005</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1033" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1033" t="n">
+        <v>23</v>
+      </c>
+      <c r="G1033" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1033" t="inlineStr">
+        <is>
+          <t>23/28</t>
+        </is>
+      </c>
+      <c r="I1033" s="5" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="J1033" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1033" t="n">
+        <v>37873147</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Lundi</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1034" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1034" t="n">
+        <v>10</v>
+      </c>
+      <c r="G1034" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1034" t="inlineStr">
+        <is>
+          <t>10/36</t>
+        </is>
+      </c>
+      <c r="I1034" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1034" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1034" t="n">
+        <v>36929042</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1028"/>
+  <autoFilter ref="A1:K1034"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-09)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1034</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1041</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1034"/>
+  <dimension ref="A1:K1041"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49073,8 +49073,337 @@
         <v>36929042</v>
       </c>
     </row>
+    <row r="1035">
+      <c r="A1035" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1035" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1035" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1035" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I1035" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J1035" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1035" t="n">
+        <v>36321369</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1036" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1036" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1036" t="inlineStr">
+        <is>
+          <t>19/28</t>
+        </is>
+      </c>
+      <c r="I1036" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J1036" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1036" t="n">
+        <v>40188418</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1037" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1037" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I1037" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1037" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1037" t="n">
+        <v>36929168</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1038" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1038" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1038" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1038" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1038" t="n">
+        <v>36298248</v>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Faustine CHOPIN</t>
+        </is>
+      </c>
+      <c r="F1039" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1039" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1039" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1039" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1039" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1039" t="n">
+        <v>36297693</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>Guided Session  (English version)</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>Théodore Zacchée</t>
+        </is>
+      </c>
+      <c r="F1040" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1040" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1040" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I1040" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1040" t="n">
+        <v>36298055</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Mardi</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1041" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1041" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1041" t="inlineStr">
+        <is>
+          <t>4/36</t>
+        </is>
+      </c>
+      <c r="I1041" s="4" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1041" t="n">
+        <v>40188451</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1034"/>
+  <autoFilter ref="A1:K1041"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-10)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1041</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1047</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1041"/>
+  <dimension ref="A1:K1047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49402,8 +49402,290 @@
         <v>40188451</v>
       </c>
     </row>
+    <row r="1042">
+      <c r="A1042" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Alice Dunoyer</t>
+        </is>
+      </c>
+      <c r="F1042" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1042" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1042" t="inlineStr">
+        <is>
+          <t>9/28</t>
+        </is>
+      </c>
+      <c r="I1042" s="4" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1042" t="n">
+        <v>36321418</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1043" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1043" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I1043" s="5" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1043" t="n">
+        <v>36929300</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1044" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1044" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1044" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1044" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1044" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1044" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1044" t="n">
+        <v>36298349</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1045" t="inlineStr">
+        <is>
+          <t>Pauline Ramon</t>
+        </is>
+      </c>
+      <c r="F1045" t="n">
+        <v>13</v>
+      </c>
+      <c r="G1045" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1045" t="inlineStr">
+        <is>
+          <t>13/28</t>
+        </is>
+      </c>
+      <c r="I1045" s="4" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="J1045" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1045" t="n">
+        <v>36298390</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1046" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1046" t="n">
+        <v>25</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1046" t="inlineStr">
+        <is>
+          <t>25/28</t>
+        </is>
+      </c>
+      <c r="I1046" s="3" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="J1046" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1046" t="n">
+        <v>36298587</v>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Mercredi</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1047" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1047" t="n">
+        <v>7</v>
+      </c>
+      <c r="G1047" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1047" t="inlineStr">
+        <is>
+          <t>7/36</t>
+        </is>
+      </c>
+      <c r="I1047" s="4" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="J1047" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1047" t="n">
+        <v>40189909</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1041"/>
+  <autoFilter ref="A1:K1047"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-11)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1047</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1060</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1047"/>
+  <dimension ref="A1:K1060"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49684,8 +49684,619 @@
         <v>40189909</v>
       </c>
     </row>
+    <row r="1048">
+      <c r="A1048" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1048" t="inlineStr">
+        <is>
+          <t>Cécile Penager</t>
+        </is>
+      </c>
+      <c r="F1048" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1048" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1048" t="inlineStr">
+        <is>
+          <t>0/28</t>
+        </is>
+      </c>
+      <c r="I1048" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1048" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1048" t="n">
+        <v>37090014</v>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1049" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1049" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1049" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1049" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1049" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1049" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1049" t="n">
+        <v>42435129</v>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1050" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1050" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1050" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1050" t="inlineStr">
+        <is>
+          <t>1/7</t>
+        </is>
+      </c>
+      <c r="I1050" s="4" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="J1050" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1050" t="n">
+        <v>37230122</v>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1051" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1051" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1051" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1051" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1051" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1051" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1051" t="n">
+        <v>37230158</v>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1052" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1052" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1052" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1052" t="inlineStr">
+        <is>
+          <t>2/7</t>
+        </is>
+      </c>
+      <c r="I1052" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J1052" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1052" t="n">
+        <v>37090972</v>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1053" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1053" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1053" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1053" t="inlineStr">
+        <is>
+          <t>0/7</t>
+        </is>
+      </c>
+      <c r="I1053" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1053" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1053" t="n">
+        <v>42430589</v>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1054" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1054" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1054" t="n">
+        <v>7</v>
+      </c>
+      <c r="H1054" t="inlineStr">
+        <is>
+          <t>5/7</t>
+        </is>
+      </c>
+      <c r="I1054" s="5" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="J1054" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1054" t="n">
+        <v>42431392</v>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1055" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1055" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1055" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1055" t="inlineStr">
+        <is>
+          <t>6/28</t>
+        </is>
+      </c>
+      <c r="I1055" s="4" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="J1055" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1055" t="n">
+        <v>36321569</v>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1056" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1056" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1056" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1056" t="inlineStr">
+        <is>
+          <t>6/18</t>
+        </is>
+      </c>
+      <c r="I1056" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1056" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1056" t="n">
+        <v>36929391</v>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1057" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1057" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1057" t="n">
+        <v>18</v>
+      </c>
+      <c r="H1057" t="inlineStr">
+        <is>
+          <t>5/18</t>
+        </is>
+      </c>
+      <c r="I1057" s="4" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="J1057" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1057" t="n">
+        <v>36298764</v>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr">
+        <is>
+          <t>Nina Petitjean</t>
+        </is>
+      </c>
+      <c r="F1058" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1058" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1058" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1058" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1058" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1058" t="n">
+        <v>36298818</v>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr">
+        <is>
+          <t>Prosper MATUSSIERE</t>
+        </is>
+      </c>
+      <c r="F1059" t="n">
+        <v>18</v>
+      </c>
+      <c r="G1059" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1059" t="inlineStr">
+        <is>
+          <t>18/28</t>
+        </is>
+      </c>
+      <c r="I1059" s="5" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="J1059" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1059" t="n">
+        <v>36298871</v>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Jeudi</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1060" t="n">
+        <v>12</v>
+      </c>
+      <c r="G1060" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1060" t="inlineStr">
+        <is>
+          <t>12/36</t>
+        </is>
+      </c>
+      <c r="I1060" s="4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="J1060" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1060" t="n">
+        <v>40189974</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1047"/>
+  <autoFilter ref="A1:K1060"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Scrap quotidien automatique (2026-09-12)
</commit_message>
<xml_diff>
--- a/reset_seances.xlsx
+++ b/reset_seances.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Seances" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1060</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Seances'!$A$1:$K$1072</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1060"/>
+  <dimension ref="A1:K1072"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50295,8 +50295,572 @@
         <v>40189974</v>
       </c>
     </row>
+    <row r="1061">
+      <c r="A1061" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr">
+        <is>
+          <t>Leonore Chapin</t>
+        </is>
+      </c>
+      <c r="F1061" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1061" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1061" t="inlineStr">
+        <is>
+          <t>14/28</t>
+        </is>
+      </c>
+      <c r="I1061" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J1061" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1061" t="n">
+        <v>36319507</v>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1062" t="n">
+        <v>9</v>
+      </c>
+      <c r="G1062" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1062" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="I1062" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1062" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1062" t="n">
+        <v>36320064</v>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1063" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1063" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1063" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1063" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1063" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1063" t="n">
+        <v>36320665</v>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1064" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1064" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1064" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1064" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1064" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1064" t="n">
+        <v>42881975</v>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1065" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1065" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1065" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1065" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1065" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1065" t="n">
+        <v>42881983</v>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1066" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1066" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1066" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+      <c r="I1066" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J1066" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1066" t="n">
+        <v>42881985</v>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1067" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1067" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1067" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1067" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1067" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1067" t="n">
+        <v>42882039</v>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1068" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1068" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1068" t="inlineStr">
+        <is>
+          <t>0/10</t>
+        </is>
+      </c>
+      <c r="I1068" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J1068" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1068" t="n">
+        <v>42882040</v>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>Quiet Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1069" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1069" t="n">
+        <v>10</v>
+      </c>
+      <c r="H1069" t="inlineStr">
+        <is>
+          <t>4/10</t>
+        </is>
+      </c>
+      <c r="I1069" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="J1069" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1069" t="n">
+        <v>42882043</v>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>Guided Session</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr">
+        <is>
+          <t>Gautier Lacointa</t>
+        </is>
+      </c>
+      <c r="F1070" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1070" t="n">
+        <v>28</v>
+      </c>
+      <c r="H1070" t="inlineStr">
+        <is>
+          <t>19/28</t>
+        </is>
+      </c>
+      <c r="I1070" s="5" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="J1070" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1070" t="n">
+        <v>36320898</v>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1071" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1071" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1071" t="inlineStr">
+        <is>
+          <t>14/36</t>
+        </is>
+      </c>
+      <c r="I1071" s="4" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="J1071" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1071" t="n">
+        <v>36893835</v>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Vendredi</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>Social Free-Flow</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr">
+        <is>
+          <t>Free Flow</t>
+        </is>
+      </c>
+      <c r="F1072" t="n">
+        <v>6</v>
+      </c>
+      <c r="G1072" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1072" t="inlineStr">
+        <is>
+          <t>6/36</t>
+        </is>
+      </c>
+      <c r="I1072" s="4" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="J1072" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="K1072" t="n">
+        <v>36893901</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1060"/>
+  <autoFilter ref="A1:K1072"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>